<commit_message>
Fixed the Bugs preventing the Test Execution and Reporting
</commit_message>
<xml_diff>
--- a/src/test/resources/data/testData.xlsx
+++ b/src/test/resources/data/testData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Environment_Collection\Intellij_Env\SeleniumTestFramework\src\test\resources\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Environments\Intellij\Selenium-Test-Framework\src\test\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44660CEB-F94F-4E8C-9CEE-F8484129A586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A3AC5D0-D749-4A89-9596-D86ECA95AEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestSuite" sheetId="3" r:id="rId1"/>
@@ -22,6 +22,9 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -420,12 +423,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{441ED292-DA54-48C6-B808-307C6EE8D48C}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
@@ -433,7 +436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -441,7 +444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -449,7 +452,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -465,13 +468,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -482,7 +485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -493,7 +496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -512,15 +515,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9C39480-F02B-40BC-AAFB-DAA923AC03BA}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -537,7 +540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -563,16 +566,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC3977DC-0C87-46C4-8425-FF285ED595B4}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -586,7 +589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>

</xml_diff>